<commit_message>
vieux trucs a synchroniser
</commit_message>
<xml_diff>
--- a/files/Excel/Solution_Portes_Couple.xlsx
+++ b/files/Excel/Solution_Portes_Couple.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/talboth/Research/Hugues/Site_Web/hugues-talbot.github.io/files/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E18C906-CA12-AB4A-AB5B-090926F8EF52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6686D35-BF20-7E4F-8B2E-B5B73CF58591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="13900" activeTab="2" xr2:uid="{28C339B6-E22C-214F-8EAC-64B6F351B033}"/>
   </bookViews>
@@ -172,7 +172,8 @@
     <definedName name="solver_ver" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">2</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -184,6 +185,7 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>

</xml_diff>